<commit_message>
Resolve URBAN COTTON SKUs from ACTX1 sales database
When MANUFACTURADO has no finished Urban Cotton product, match by
gender, size, and color against urban_cotton_ACTX1.xlsx using the
most frequent SKU per combination.

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/por_ajuste_sku_con_sku.xlsx
+++ b/output/por_ajuste_sku_con_sku.xlsx
@@ -4574,15 +4574,23 @@
           <t>AZUL MARINO</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>TALGTACA12TXL</t>
+        </is>
+      </c>
       <c r="F102" t="n">
         <v>1</v>
       </c>
       <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr"/>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>URBAN COTTON OVERSIZED OUTSIDE</t>
+        </is>
+      </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>product_not_found</t>
+          <t>ok_urban_cotton</t>
         </is>
       </c>
     </row>
@@ -4607,15 +4615,23 @@
           <t>AZUL MARINO</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>TALGTACA12TM</t>
+        </is>
+      </c>
       <c r="F103" t="n">
         <v>1</v>
       </c>
       <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>URBAN COTTON OVERSIZED OUTSIDE</t>
+        </is>
+      </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>product_not_found</t>
+          <t>ok_urban_cotton</t>
         </is>
       </c>
     </row>
@@ -4640,15 +4656,23 @@
           <t>AZUL MARINO</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>TALGTACA12TL</t>
+        </is>
+      </c>
       <c r="F104" t="n">
         <v>1</v>
       </c>
       <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>URBAN COTTON OVERSIZED OUTSIDE</t>
+        </is>
+      </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>product_not_found</t>
+          <t>ok_urban_cotton</t>
         </is>
       </c>
     </row>
@@ -4673,15 +4697,23 @@
           <t>AZUL MARINO</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>TALGTACA12TXS</t>
+        </is>
+      </c>
       <c r="F105" t="n">
         <v>1</v>
       </c>
       <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr"/>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>URBAN COTTON OVERSIZED OUTSIDE</t>
+        </is>
+      </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>product_not_found</t>
+          <t>ok_urban_cotton</t>
         </is>
       </c>
     </row>
@@ -4706,15 +4738,23 @@
           <t>AZUL MARINO</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>TALGTADA12TS</t>
+        </is>
+      </c>
       <c r="F106" t="n">
         <v>1</v>
       </c>
       <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>URBAN COTTON TOP SAY YES</t>
+        </is>
+      </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>product_not_found</t>
+          <t>ok_urban_cotton</t>
         </is>
       </c>
     </row>
@@ -4739,15 +4779,23 @@
           <t>AZUL MARINO</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>TALGTADA12TL</t>
+        </is>
+      </c>
       <c r="F107" t="n">
         <v>1</v>
       </c>
       <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>URBAN COTTON TOP SAY YES</t>
+        </is>
+      </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>product_not_found</t>
+          <t>ok_urban_cotton</t>
         </is>
       </c>
     </row>
@@ -4772,15 +4820,23 @@
           <t>AZUL MARINO</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>TALGTADA12TM</t>
+        </is>
+      </c>
       <c r="F108" t="n">
         <v>1</v>
       </c>
       <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>URBAN COTTON TOP SAY YES</t>
+        </is>
+      </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>product_not_found</t>
+          <t>ok_urban_cotton</t>
         </is>
       </c>
     </row>
@@ -10454,7 +10510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10507,22 +10563,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">URBAN COTTON </t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>XL</t>
-        </is>
+          <t>SHORT SPORT</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>16</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CABALLERO</t>
+          <t>KIDS</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>AZUL MARINO</t>
+          <t>GRIS C</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -10530,32 +10584,34 @@
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>SHORT SPORT</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>product_not_found</t>
+          <t>talla_not_found</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">URBAN COTTON </t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
+          <t>SHORT SPORT</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>16</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CABALLERO</t>
+          <t>KIDS</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>AZUL MARINO</t>
+          <t>BLANCO</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -10563,243 +10619,12 @@
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>SHORT SPORT</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
-        <is>
-          <t>product_not_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">URBAN COTTON </t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CABALLERO</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>AZUL MARINO</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>product_not_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">URBAN COTTON </t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>XS</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CABALLERO</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>AZUL MARINO</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>product_not_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">URBAN COTTON </t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>DAMA</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>AZUL MARINO</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>product_not_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">URBAN COTTON </t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>DAMA</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>AZUL MARINO</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>product_not_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">URBAN COTTON </t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>DAMA</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>AZUL MARINO</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>product_not_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>SHORT SPORT</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>16</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>KIDS</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>GRIS C</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>SHORT SPORT</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>talla_not_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>SHORT SPORT</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>16</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>KIDS</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>BLANCO</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>SHORT SPORT</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
         <is>
           <t>talla_not_found</t>
         </is>

</xml_diff>